<commit_message>
ground_truth_review update + parse_tracker_log creation
</commit_message>
<xml_diff>
--- a/output_fish_tracker/ground_truth_review/ground_truth_review_2026_07_06_1931.xlsx
+++ b/output_fish_tracker/ground_truth_review/ground_truth_review_2026_07_06_1931.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/govinda-dashugolienart/Documents/Github_HD/AquaMind/output_fish_tracker/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/govinda-dashugolienart/Documents/Github_HD/AquaMind/output_fish_tracker/ground_truth_review/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{954EFE0D-FDE0-E248-9C7B-DD2D79D22B27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{172BCF68-9A31-8643-94F0-5E78D67EE10A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16660" xr2:uid="{6449AD96-D7A3-8545-9628-8683DD62E81D}"/>
+    <workbookView xWindow="28800" yWindow="-860" windowWidth="38400" windowHeight="21600" xr2:uid="{6449AD96-D7A3-8545-9628-8683DD62E81D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="database" sheetId="1" r:id="rId1"/>
+    <sheet name="legend" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="41">
   <si>
     <t>run_name</t>
   </si>
@@ -54,13 +55,139 @@
   </si>
   <si>
     <t>error_type</t>
+  </si>
+  <si>
+    <t>stage5_tracker_IMG_2349_as_3r_4r_5r_8c_2026_07_06_1853</t>
+  </si>
+  <si>
+    <t>crossing</t>
+  </si>
+  <si>
+    <t>Fish got close/overlapped but did not actually cross paths; tracker incorrectly swapped their IDs</t>
+  </si>
+  <si>
+    <t>missing_track</t>
+  </si>
+  <si>
+    <t>Box briefly attaches to the fish's own reflection instead of the real fish; typically self-corrects within a few frames</t>
+  </si>
+  <si>
+    <t>reflection_confusion</t>
+  </si>
+  <si>
+    <t>occlusion_recovery</t>
+  </si>
+  <si>
+    <t>Fish 1 emerged from occlusion at 3858, grabbed Fish 2's tag at 3861; IDs flickered back and forth repeatedly (3871, 3877, 3890...) while Fish 1's original track sat "lost" near the occlusion spot the whole time; stabilized only at 3989 when Fish 1 happened to swim back near where it first vanishe</t>
+  </si>
+  <si>
+    <t>Fish got close/overlapped but did not actually cross paths; tracker incorrectly swapped their IDs. A lot of flickering but evenually wrong tag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">occlusion_recovery	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7290	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7346	</t>
+  </si>
+  <si>
+    <t>As the long-"lost" Fish 4 track drifted close to the confirmed Fish 2, it briefly stole Fish 2's tag (Fish 2 went untagged for a moment), then snapped back to the correct assignment by ~7332. The real Fish 4 body stayed untagged until it happened to swim back near where its own tag was originally dropped, finally reclaiming "Fish 4" at frame 7346.</t>
+  </si>
+  <si>
+    <t>run_id</t>
+  </si>
+  <si>
+    <t>What it means</t>
+  </si>
+  <si>
+    <t>How to spot it</t>
+  </si>
+  <si>
+    <t>Cross-checked against</t>
+  </si>
+  <si>
+    <t>Two fish's boxes closed in/overlapped, and the tracker assigned the wrong IDs after separating (or failed to swap when it should have)</t>
+  </si>
+  <si>
+    <t>Two boxes converge, briefly merge/overlap, then separate — compare each fish's color/shade before vs. after to judge correctness</t>
+  </si>
+  <si>
+    <t>A dashed "lost" ID reappears on a different, wrong fish; or two IDs swap/flicker around a reappearance</t>
+  </si>
+  <si>
+    <t>Fish has zero box anywhere on it — OR a dashed box is frozen at a stale, old position while the real fish is visible elsewhere with nothing drawn on it</t>
+  </si>
+  <si>
+    <t>No box at all near the visible fish; or a "lost" box stuck in one place while the fish has clearly swum away from it</t>
+  </si>
+  <si>
+    <t>Nothing — human-only</t>
+  </si>
+  <si>
+    <t>Box briefly attaches to a reflection (own or another fish's) instead of the real fish</t>
+  </si>
+  <si>
+    <t>Tag lands on a mirror image / faint duplicate near glass or waterline; usually self-corrects within a few frames</t>
+  </si>
+  <si>
+    <r>
+      <t>A fish reappearing after being genuinely hidden (behind plant/pipe, or sitting "lost") gets matched onto the </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>wrong</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> physical body</t>
+    </r>
+  </si>
+  <si>
+    <t>Step 2's parsed log (Crossing started / IDs swapped / no swap)</t>
+  </si>
+  <si>
+    <t>Step 2's parsed log (Fish X recovered after N missing frames)</t>
+  </si>
+  <si>
+    <t>ish clearly visible on right side but tracker drew no box at all -&gt; not even "lost" , for ~10 seconds</t>
+  </si>
+  <si>
+    <t>fish clearly visible on right side but tracker drew no box at all -&gt; not even "lost" for 90 frames</t>
+  </si>
+  <si>
+    <t>Fish 2 recovered from occlusion but matched onto the nearest detection instead of its own body -&gt; landed on Fish 1 (untagged at the time). Recovery matching is position-only, no identity check.</t>
+  </si>
+  <si>
+    <t>fish clearly visible on right side but tracker drew no box at all -&gt; not even "lost" for at least 600 frames but when the fish passes again where the tag got lost it regains its tag</t>
+  </si>
+  <si>
+    <t>Fish 2 emerged from behind the pipe at ~5581 and immediately full-swapped with the nearby Fish 4 (not a one-sided grab like before -&gt; both tags flipped simultaneously: real Fish 4's body became labeled "2", real Fish 2's body became labeled "4"). Mislabeling persisted unnoticed through 5665. Got messier ~5793 (tag lost again). At 6217, whichever fish was wearing tag "2" handed it off again to a different untagged fish, losing its own tag a second time. Finally stabilized at 6417 when the long-untagged fish happened to swim back near where a tag was originally dropped and reclaimed it as "Fish 4." ~840 frames (14s) of instability from one triggering event.</t>
+  </si>
+  <si>
+    <t>In the middle of the above chaos, Fish 2's tag briefly jumped onto a reflection (~5812), then returned to the real fish by 5846 -&gt; a self-contained sub-glitch nested inside the larger occlusion_recovery incident.</t>
+  </si>
+  <si>
+    <t>Dashed "lost" box stayed frozen at Fish 4's last known position while the real fish was clearly visible swimming elsewhere in open water -&gt; zero box on its actual position for the whole window, until it gained a (wrong) tag at 7290</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -69,13 +196,33 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10.8"/>
-      <color rgb="FF88C0D0"/>
-      <name val="Courier New"/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -88,8 +235,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -112,37 +271,44 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -478,203 +644,520 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F57440F-245A-BC4D-AD68-D8B02E510501}">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" customWidth="1"/>
-    <col min="2" max="3" width="20" customWidth="1"/>
-    <col min="4" max="5" width="23.6640625" customWidth="1"/>
-    <col min="6" max="6" width="25" customWidth="1"/>
+    <col min="1" max="1" width="27.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="63.33203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.1640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="11.5" style="2" customWidth="1"/>
+    <col min="6" max="6" width="23.6640625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="70.33203125" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:7" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="4"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="2"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="2"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="2"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
+    </row>
+    <row r="2" spans="1:7" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="8">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="4">
+        <v>790</v>
+      </c>
+      <c r="D2" s="4">
+        <v>860</v>
+      </c>
+      <c r="E2" s="4">
+        <v>1.3</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="8">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="4">
+        <v>1178</v>
+      </c>
+      <c r="D3" s="4">
+        <v>1264</v>
+      </c>
+      <c r="E3" s="4">
+        <v>1.3</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="8">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1744</v>
+      </c>
+      <c r="D4" s="4">
+        <v>1805</v>
+      </c>
+      <c r="E4" s="4">
+        <v>2.4</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="8">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="4">
+        <v>1969</v>
+      </c>
+      <c r="D5" s="4">
+        <v>2311</v>
+      </c>
+      <c r="E5" s="4">
+        <v>1</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="8">
+        <v>1</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="4">
+        <v>2521</v>
+      </c>
+      <c r="D6" s="4">
+        <v>2565</v>
+      </c>
+      <c r="E6" s="4">
+        <v>2</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="8">
+        <v>1</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="4">
+        <v>2600</v>
+      </c>
+      <c r="D7" s="4">
+        <v>2690</v>
+      </c>
+      <c r="E7" s="4">
+        <v>1</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="8">
+        <v>1</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="4">
+        <v>2673</v>
+      </c>
+      <c r="D8" s="4">
+        <v>2686</v>
+      </c>
+      <c r="E8" s="4">
+        <v>2</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="8">
+        <v>1</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="4">
+        <v>2693</v>
+      </c>
+      <c r="D9" s="4">
+        <v>3300</v>
+      </c>
+      <c r="E9" s="4">
+        <v>1</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="8">
+        <v>1</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="4">
+        <v>3529</v>
+      </c>
+      <c r="D10" s="4">
+        <v>3549</v>
+      </c>
+      <c r="E10" s="4">
+        <v>1.2</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="97" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="8">
+        <v>1</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="7">
+        <v>3850</v>
+      </c>
+      <c r="D11" s="7">
+        <v>4000</v>
+      </c>
+      <c r="E11" s="4">
+        <v>1.2</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="8">
+        <v>1</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="4">
+        <v>4230</v>
+      </c>
+      <c r="D12" s="4">
+        <v>4351</v>
+      </c>
+      <c r="E12" s="4">
+        <v>1.2</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="8">
+        <v>1</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="4">
+        <v>4825</v>
+      </c>
+      <c r="D13" s="4">
+        <v>4849</v>
+      </c>
+      <c r="E13" s="4">
+        <v>1.4</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="8">
+        <v>1</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="4">
+        <v>5002</v>
+      </c>
+      <c r="D14" s="4">
+        <v>5074</v>
+      </c>
+      <c r="E14" s="4">
+        <v>1.2</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="213" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="8">
+        <v>1</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="4">
+        <v>5570</v>
+      </c>
+      <c r="D15" s="4">
+        <v>6417</v>
+      </c>
+      <c r="E15" s="4">
+        <v>2.4</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="8">
+        <v>1</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="4">
+        <v>5805</v>
+      </c>
+      <c r="D16" s="4">
+        <v>5850</v>
+      </c>
+      <c r="E16" s="4">
+        <v>2</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="76" x14ac:dyDescent="0.2">
+      <c r="A17" s="8">
+        <v>1</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="4">
+        <v>7150</v>
+      </c>
+      <c r="D17" s="4">
+        <v>7300</v>
+      </c>
+      <c r="E17" s="4">
+        <v>4</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="161" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="8">
+        <v>1</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" s="4">
+        <v>2.4</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D1667ED-DF75-C943-B716-1237CD458FA3}">
+  <dimension ref="B2:E6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" style="10"/>
+    <col min="2" max="2" width="27.1640625" style="10" customWidth="1"/>
+    <col min="3" max="3" width="51.5" style="10" customWidth="1"/>
+    <col min="4" max="4" width="130.5" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="69" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="10.83203125" style="10"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="B3" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="B4" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="B5" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="B6" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>28</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>